<commit_message>
feat: initialize project structure with core components, documentation, data seeds, and build automation tools
</commit_message>
<xml_diff>
--- a/deliverables/VYTAL_House_Operations_Workbook.xlsx
+++ b/deliverables/VYTAL_House_Operations_Workbook.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R46198a993afd42fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R2d28ee5284b949d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue_Model" sheetId="3" r:id="Rbfb10abd62b24aca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendor_Outreach" sheetId="4" r:id="R5ae4418a98e94a12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Social_Calendar" sheetId="5" r:id="R2ddc340b64f4473a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources_Audit" sheetId="6" r:id="Rd77d618328bc407c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="7" r:id="Re19cc45fbd2449a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re2634055cf834c66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R80467c2ca91144ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue_Model" sheetId="3" r:id="R093cec1e6b7344a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendor_Outreach" sheetId="4" r:id="R295bef69c25d4d73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Social_Calendar" sheetId="5" r:id="R6993f3debafd44ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources_Audit" sheetId="6" r:id="R4d98a0067b3f4d18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Readiness" sheetId="7" r:id="Rba455352eaef44b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="Rc314635a57e943a5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -330,7 +331,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb9843e4128bc48d4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7e39a8eaa26e4652"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -589,10 +590,10 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="11" t="str">
-        <x:v>Target quality gate</x:v>
-      </x:c>
-      <x:c r="B4" s="11" t="n">
-        <x:v>97</x:v>
+        <x:v>Target location</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="str">
+        <x:v>6000 Merriweather Drive, Columbia, MD 21044</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
         <x:v>Core</x:v>
@@ -606,10 +607,10 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="11" t="str">
-        <x:v>Current package score</x:v>
+        <x:v>Target quality gate</x:v>
       </x:c>
       <x:c r="B5" s="11" t="n">
-        <x:v>100</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="D5" s="11" t="str">
         <x:v>Elite</x:v>
@@ -623,35 +624,43 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="11" t="str">
+        <x:v>Current package score</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="str">
+        <x:v>Black</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F6" s="12" t="n">
+        <x:v>74950</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="11" t="str">
         <x:v>Modeled membership MRR</x:v>
       </x:c>
-      <x:c r="B6" s="12" t="n">
+      <x:c r="B7" s="12" t="n">
         <x:f>Revenue_Model!D7</x:f>
         <x:v>179700</x:v>
       </x:c>
-      <x:c r="D6" s="11" t="str">
-        <x:v>Black</x:v>
-      </x:c>
-      <x:c r="E6" s="11" t="n">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="F6" s="12" t="n">
-        <x:v>74950</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="11" t="str">
-        <x:v>Vendor quote targets</x:v>
-      </x:c>
-      <x:c r="B7" s="11" t="n">
-        <x:v>4</x:v>
-      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="11" t="str">
+        <x:v>Vendor quote targets</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="11" t="str">
         <x:v>Draft social posts</x:v>
       </x:c>
-      <x:c r="B8" s="11" t="n">
+      <x:c r="B9" s="11" t="n">
         <x:v>10</x:v>
       </x:c>
     </x:row>
@@ -660,7 +669,7 @@
     <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R828d636244c546e7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcb95d657e6746a0"/>
 </x:worksheet>
 </file>
 
@@ -1565,6 +1574,320 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="36.66999816894531" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="25.5" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Project Readiness</x:v>
+      </x:c>
+      <x:c r="B1" s="4" t="str">
+        <x:v>Project Readiness</x:v>
+      </x:c>
+      <x:c r="C1" s="4" t="str">
+        <x:v>Project Readiness</x:v>
+      </x:c>
+      <x:c r="D1" s="4" t="str">
+        <x:v>Project Readiness</x:v>
+      </x:c>
+      <x:c r="E1" s="4" t="str">
+        <x:v>Project Readiness</x:v>
+      </x:c>
+      <x:c r="F1" s="4" t="str">
+        <x:v>Project Readiness</x:v>
+      </x:c>
+      <x:c r="G1" s="4" t="str">
+        <x:v>Project Readiness</x:v>
+      </x:c>
+      <x:c r="H1" s="4" t="str">
+        <x:v>Project Readiness</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="7" t="str">
+        <x:v>Record</x:v>
+      </x:c>
+      <x:c r="B3" s="7" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="C3" s="7" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="D3" s="7" t="str">
+        <x:v>Gate</x:v>
+      </x:c>
+      <x:c r="E3" s="7" t="str">
+        <x:v>Control</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="11" t="str">
+        <x:v>Confirm ownership economics</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="str">
+        <x:v>owner</x:v>
+      </x:c>
+      <x:c r="C4" s="11" t="str">
+        <x:v>approval-needed</x:v>
+      </x:c>
+      <x:c r="D4" s="11" t="str">
+        <x:v>Formation</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="str">
+        <x:v>Before formation filings</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="11" t="str">
+        <x:v>Confirm Merriweather lease, zoning, utilities, and tenant improvements</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
+        <x:v>operations</x:v>
+      </x:c>
+      <x:c r="C5" s="11" t="str">
+        <x:v>approval-needed</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="str">
+        <x:v>Lease</x:v>
+      </x:c>
+      <x:c r="E5" s="11" t="str">
+        <x:v>Before vendor deposits</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="11" t="str">
+        <x:v>Secure medical director letter of intent</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
+        <x:v>clinical</x:v>
+      </x:c>
+      <x:c r="C6" s="11" t="str">
+        <x:v>approval-needed</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="str">
+        <x:v>Medical</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="str">
+        <x:v>Before clinical service pre-sale</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="11" t="str">
+        <x:v>Request formal equipment quotes</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str">
+        <x:v>operations</x:v>
+      </x:c>
+      <x:c r="C7" s="11" t="str">
+        <x:v>quote-needed</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="str">
+        <x:v>After owner approval to contact vendors</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="11" t="str">
+        <x:v>Manifest Firebase staging project</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="str">
+        <x:v>admin</x:v>
+      </x:c>
+      <x:c r="C8" s="11" t="str">
+        <x:v>ready-draft</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="str">
+        <x:v>Technology</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="str">
+        <x:v>After Google Cloud project approval</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="11" t="str">
+        <x:v>Create governed Google Cloud file vault plan</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="str">
+        <x:v>admin</x:v>
+      </x:c>
+      <x:c r="C9" s="11" t="str">
+        <x:v>ready-draft</x:v>
+      </x:c>
+      <x:c r="D9" s="11" t="str">
+        <x:v>Document vault</x:v>
+      </x:c>
+      <x:c r="E9" s="11" t="str">
+        <x:v>Before live document import</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="11" t="str">
+        <x:v>Medical claims not reviewed</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="str">
+        <x:v>marketing</x:v>
+      </x:c>
+      <x:c r="C10" s="11" t="str">
+        <x:v>open</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E10" s="11" t="str">
+        <x:v>Approved claims library and clinical/counsel review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="11" t="str">
+        <x:v>Equipment delays</x:v>
+      </x:c>
+      <x:c r="B11" s="11" t="str">
+        <x:v>operations</x:v>
+      </x:c>
+      <x:c r="C11" s="11" t="str">
+        <x:v>open</x:v>
+      </x:c>
+      <x:c r="D11" s="11" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E11" s="11" t="str">
+        <x:v>Multiple vendor quotes and lead-time tracking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="11" t="str">
+        <x:v>Data breach</x:v>
+      </x:c>
+      <x:c r="B12" s="11" t="str">
+        <x:v>admin</x:v>
+      </x:c>
+      <x:c r="C12" s="11" t="str">
+        <x:v>open</x:v>
+      </x:c>
+      <x:c r="D12" s="11" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E12" s="11" t="str">
+        <x:v>MFA, RBAC, encryption, audit logs, and no PHI in prototype</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="11" t="str">
+        <x:v>Founder deadlock</x:v>
+      </x:c>
+      <x:c r="B13" s="11" t="str">
+        <x:v>owner</x:v>
+      </x:c>
+      <x:c r="C13" s="11" t="str">
+        <x:v>open</x:v>
+      </x:c>
+      <x:c r="D13" s="11" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E13" s="11" t="str">
+        <x:v>Operating agreement deadlock and buy-sell mechanics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="11" t="str">
+        <x:v>GitHub repository</x:v>
+      </x:c>
+      <x:c r="B14" s="11" t="str">
+        <x:v>admin</x:v>
+      </x:c>
+      <x:c r="C14" s="11" t="str">
+        <x:v>connected-local</x:v>
+      </x:c>
+      <x:c r="D14" s="11" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="E14" s="11" t="str">
+        <x:v>Push allowed only for VYTAL-scoped code and docs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="11" t="str">
+        <x:v>Firebase staging</x:v>
+      </x:c>
+      <x:c r="B15" s="11" t="str">
+        <x:v>admin</x:v>
+      </x:c>
+      <x:c r="C15" s="11" t="str">
+        <x:v>ready-draft</x:v>
+      </x:c>
+      <x:c r="D15" s="11" t="str">
+        <x:v>Firebase</x:v>
+      </x:c>
+      <x:c r="E15" s="11" t="str">
+        <x:v>Owner approval, Firebase project, custom claims, App Check, and rules deploy</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="11" t="str">
+        <x:v>Google Cloud file vault</x:v>
+      </x:c>
+      <x:c r="B16" s="11" t="str">
+        <x:v>admin</x:v>
+      </x:c>
+      <x:c r="C16" s="11" t="str">
+        <x:v>ready-draft</x:v>
+      </x:c>
+      <x:c r="D16" s="11" t="str">
+        <x:v>Google Cloud</x:v>
+      </x:c>
+      <x:c r="E16" s="11" t="str">
+        <x:v>IAM roles, retention rules, encryption, professional review folders, and owner approval</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="11" t="str">
+        <x:v>Notion importables</x:v>
+      </x:c>
+      <x:c r="B17" s="11" t="str">
+        <x:v>operations</x:v>
+      </x:c>
+      <x:c r="C17" s="11" t="str">
+        <x:v>ready-draft</x:v>
+      </x:c>
+      <x:c r="D17" s="11" t="str">
+        <x:v>Notion</x:v>
+      </x:c>
+      <x:c r="E17" s="11" t="str">
+        <x:v>No live workspace mutation until approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="11" t="str">
+        <x:v>Figma design handoff</x:v>
+      </x:c>
+      <x:c r="B18" s="11" t="str">
+        <x:v>marketing</x:v>
+      </x:c>
+      <x:c r="C18" s="11" t="str">
+        <x:v>ready-draft</x:v>
+      </x:c>
+      <x:c r="D18" s="11" t="str">
+        <x:v>Figma</x:v>
+      </x:c>
+      <x:c r="E18" s="11" t="str">
+        <x:v>No live Figma file creation until approved</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
       <x:c r="A1" s="4" t="str">
@@ -1725,13 +2048,13 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="11" t="str">
-        <x:v>No live external mutation</x:v>
+        <x:v>Launch goals</x:v>
       </x:c>
       <x:c r="B9" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C9" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D9" s="11" t="n">
         <x:f>B9-C9</x:f>
@@ -1741,20 +2064,42 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F9" s="11" t="str">
-        <x:f>IF(B9=C9,"OK","FAIL")</x:f>
+        <x:f>IF(B9&gt;=C9,"OK","FAIL")</x:f>
         <x:v>OK</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="11" t="str">
+        <x:v>No live external mutation</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="n">
+        <x:f>B10-C10</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F10" s="11" t="str">
+        <x:f>IF(B10=C10,"OK","FAIL")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="11" t="str">
         <x:v>Model status</x:v>
       </x:c>
-      <x:c r="B10" s="11" t="str"/>
-      <x:c r="C10" s="11" t="str"/>
-      <x:c r="D10" s="11" t="str"/>
-      <x:c r="E10" s="11" t="str"/>
-      <x:c r="F10" s="11" t="str">
-        <x:f>IF(COUNTIF(F4:F9,"FAIL")=0,"OK","FAIL")</x:f>
+      <x:c r="B11" s="11" t="str"/>
+      <x:c r="C11" s="11" t="str"/>
+      <x:c r="D11" s="11" t="str"/>
+      <x:c r="E11" s="11" t="str"/>
+      <x:c r="F11" s="11" t="str">
+        <x:f>IF(COUNTIF(F4:F10,"FAIL")=0,"OK","FAIL")</x:f>
         <x:v>OK</x:v>
       </x:c>
     </x:row>

</xml_diff>